<commit_message>
Dive arreglando con la libreria threads, mejorando la vista step2
</commit_message>
<xml_diff>
--- a/LISTAS/ma/BROCHE MEDIA SOMBRA.xlsx
+++ b/LISTAS/ma/BROCHE MEDIA SOMBRA.xlsx
@@ -737,7 +737,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="34" t="n">
-        <v>45238</v>
+        <v>45239</v>
       </c>
       <c r="E1" s="4" t="n"/>
     </row>
@@ -877,18 +877,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="A1:D1"/>
     <mergeCell ref="B38:C38"/>
-    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="B29:C29"/>
     <mergeCell ref="A12:D12"/>
     <mergeCell ref="B37:C37"/>
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A10:D10"/>
     <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B29:C29"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
puliendo interfaz web, y buscador para q reselte los resultados
</commit_message>
<xml_diff>
--- a/LISTAS/ma/BROCHE MEDIA SOMBRA.xlsx
+++ b/LISTAS/ma/BROCHE MEDIA SOMBRA.xlsx
@@ -737,7 +737,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="34" t="n">
-        <v>45244</v>
+        <v>45245</v>
       </c>
       <c r="E1" s="4" t="n"/>
     </row>
@@ -877,18 +877,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="A1:D1"/>
     <mergeCell ref="B38:C38"/>
-    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="B29:C29"/>
     <mergeCell ref="A12:D12"/>
     <mergeCell ref="B37:C37"/>
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A10:D10"/>
     <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B29:C29"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
haciendo buscador con problemas
</commit_message>
<xml_diff>
--- a/LISTAS/ma/BROCHE MEDIA SOMBRA.xlsx
+++ b/LISTAS/ma/BROCHE MEDIA SOMBRA.xlsx
@@ -877,18 +877,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A10:D10"/>
     <mergeCell ref="B38:C38"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="A11:D11"/>
     <mergeCell ref="A12:D12"/>
     <mergeCell ref="B37:C37"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B39:C39"/>
     <mergeCell ref="B28:C28"/>
+    <mergeCell ref="A9:D9"/>
     <mergeCell ref="B36:C36"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B29:C29"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
a la vista pincipal se le agrego la tarea de verificar si hay archivos pendientes a subir y e intentar resubirlos
</commit_message>
<xml_diff>
--- a/LISTAS/ma/BROCHE MEDIA SOMBRA.xlsx
+++ b/LISTAS/ma/BROCHE MEDIA SOMBRA.xlsx
@@ -737,7 +737,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="34" t="n">
-        <v>45254</v>
+        <v>45255</v>
       </c>
       <c r="E1" s="4" t="n"/>
     </row>
@@ -877,18 +877,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="A1:D1"/>
     <mergeCell ref="B38:C38"/>
-    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="B29:C29"/>
     <mergeCell ref="A12:D12"/>
     <mergeCell ref="B37:C37"/>
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A10:D10"/>
     <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B29:C29"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>